<commit_message>
refact: Status column inside the content of the `notes/Notes.xlsx`
</commit_message>
<xml_diff>
--- a/notes/Notes.xlsx
+++ b/notes/Notes.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Visual_Studio_Codes\Data-Bank-System\references\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Visual_Studio_Codes\Data-Bank-System\notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4CC5D51-5974-47F0-8F51-4AF394BB52F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2DA7684-E81C-4C21-BD00-34E548B22977}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7B6336E8-B946-4BA0-8A65-45DEACE9975D}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="57">
   <si>
     <t>INDICATORS</t>
   </si>
@@ -215,9 +215,6 @@
   </si>
   <si>
     <t>same sa nasa taas ang pagkakaiba yung data sa pagmemeasure nila. PNP - Barangay, MBDA - Latitude/Longitude</t>
-  </si>
-  <si>
-    <t>ONGOING</t>
   </si>
   <si>
     <t>running average. Injury count total in any injury types and severities</t>
@@ -864,10 +861,10 @@
         <v>39</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>56</v>
+        <v>37</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="64.2" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -904,18 +901,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1063,14 +1060,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67B8CFB1-3E32-4F77-BEE9-45E50532F813}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BDD56014-E7AA-4ACA-8617-149CD20A7624}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
@@ -1082,6 +1071,14 @@
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67B8CFB1-3E32-4F77-BEE9-45E50532F813}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
feat: Update the description column from the excel file
</commit_message>
<xml_diff>
--- a/notes/Notes.xlsx
+++ b/notes/Notes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Visual_Studio_Codes\Data-Bank-System\notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2DA7684-E81C-4C21-BD00-34E548B22977}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{601B1548-C3A9-483A-BDDA-E0831A6FEF2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7B6336E8-B946-4BA0-8A65-45DEACE9975D}"/>
   </bookViews>
@@ -195,9 +195,6 @@
     <t>Sir Nico kaso nakaleave, nasa gilid siya, pwede naman daw ako gumawa muna ng initial ERD ko for that. May binigay na context sa akin si Sir Jap, naka time-based daw yung pag-track ng progress percentage ng mga master development plan and dapat tinatrack ko siya per barangay and not total barangay. Every 3 years dapat tinatrack ko yung progress percentage. Dapat din may 3 types of plans na sinasubmit bawat plan (Initial, Revised, Approved). Kung sakop pa ng range niya yung Date Range sa sinubmit na Plan, dapat updated yun</t>
   </si>
   <si>
-    <t>Hintayin or update si Ma'am Joana kung kailan makukuha yung raw data for this indicator</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">Kay Sir Jap lang ako nagtanong kaya binigyan ako ng column. Tanong mo nalang saan galing yung data na sinend niya sa akin. annually, may target pct per 3 years, pero index crime lang siya. </t>
     </r>
@@ -218,6 +215,9 @@
   </si>
   <si>
     <t>running average. Injury count total in any injury types and severities</t>
+  </si>
+  <si>
+    <t>Binigay na sa akin yung data thru email</t>
   </si>
 </sst>
 </file>
@@ -774,7 +774,7 @@
         <v>39</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="I7" s="3" t="s">
         <v>38</v>
@@ -803,7 +803,7 @@
         <v>39</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I10" s="3" t="s">
         <v>37</v>
@@ -832,7 +832,7 @@
         <v>39</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="I11" s="3" t="s">
         <v>37</v>
@@ -861,7 +861,7 @@
         <v>39</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="I12" s="3" t="s">
         <v>37</v>
@@ -901,18 +901,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1060,6 +1060,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67B8CFB1-3E32-4F77-BEE9-45E50532F813}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BDD56014-E7AA-4ACA-8617-149CD20A7624}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
@@ -1071,14 +1079,6 @@
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67B8CFB1-3E32-4F77-BEE9-45E50532F813}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Update the status of the row for the indicator `% improvement in government employee service quality`
</commit_message>
<xml_diff>
--- a/notes/Notes.xlsx
+++ b/notes/Notes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Visual_Studio_Codes\Data-Bank-System\notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{601B1548-C3A9-483A-BDDA-E0831A6FEF2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59B994F5-3F96-4AB7-935D-A75589EBCE75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7B6336E8-B946-4BA0-8A65-45DEACE9975D}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="58">
   <si>
     <t>INDICATORS</t>
   </si>
@@ -218,6 +218,9 @@
   </si>
   <si>
     <t>Binigay na sa akin yung data thru email</t>
+  </si>
+  <si>
+    <t>PACHECK KAY SIR JAP</t>
   </si>
 </sst>
 </file>
@@ -777,7 +780,7 @@
         <v>56</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>38</v>
+        <v>57</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="72" x14ac:dyDescent="0.3">
@@ -910,12 +913,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C5A14CB71E5AFD41970DCC84E250D579" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="5cb02eec2b50f308d3d8c622b39c24e6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="6aee86ec-03d1-4b31-a311-732977dc0399" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3e885d23f01897dc3817344103bdb46e" ns3:_="">
     <xsd:import namespace="6aee86ec-03d1-4b31-a311-732977dc0399"/>
@@ -1059,6 +1056,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67B8CFB1-3E32-4F77-BEE9-45E50532F813}">
   <ds:schemaRefs>
@@ -1068,22 +1071,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BDD56014-E7AA-4ACA-8617-149CD20A7624}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="6aee86ec-03d1-4b31-a311-732977dc0399"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A5169A02-7206-4788-A357-046EDE3DF615}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1099,4 +1086,20 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BDD56014-E7AA-4ACA-8617-149CD20A7624}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="6aee86ec-03d1-4b31-a311-732977dc0399"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update the status column of the Notes excel file
</commit_message>
<xml_diff>
--- a/notes/Notes.xlsx
+++ b/notes/Notes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Visual_Studio_Codes\Data-Bank-System\notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59B994F5-3F96-4AB7-935D-A75589EBCE75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE03CA87-4692-4324-A673-309992154EE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7B6336E8-B946-4BA0-8A65-45DEACE9975D}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="59">
   <si>
     <t>INDICATORS</t>
   </si>
@@ -221,6 +221,9 @@
   </si>
   <si>
     <t>PACHECK KAY SIR JAP</t>
+  </si>
+  <si>
+    <t>PACHECK KAY SIR JAP KASI NIREVISE MO ULI</t>
   </si>
 </sst>
 </file>
@@ -867,7 +870,7 @@
         <v>55</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>37</v>
+        <v>58</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="64.2" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -894,7 +897,7 @@
         <v>39</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>38</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -904,12 +907,9 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1057,15 +1057,26 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67B8CFB1-3E32-4F77-BEE9-45E50532F813}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BDD56014-E7AA-4ACA-8617-149CD20A7624}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="6aee86ec-03d1-4b31-a311-732977dc0399"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1089,17 +1100,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BDD56014-E7AA-4ACA-8617-149CD20A7624}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67B8CFB1-3E32-4F77-BEE9-45E50532F813}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="6aee86ec-03d1-4b31-a311-732977dc0399"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update the status column of the `notes/notes.xlsx`
</commit_message>
<xml_diff>
--- a/notes/Notes.xlsx
+++ b/notes/Notes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Visual_Studio_Codes\Data-Bank-System\notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE03CA87-4692-4324-A673-309992154EE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C0EEC82-6AEF-440E-AF22-DE300DC9807E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7B6336E8-B946-4BA0-8A65-45DEACE9975D}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="57">
   <si>
     <t>INDICATORS</t>
   </si>
@@ -218,12 +218,6 @@
   </si>
   <si>
     <t>Binigay na sa akin yung data thru email</t>
-  </si>
-  <si>
-    <t>PACHECK KAY SIR JAP</t>
-  </si>
-  <si>
-    <t>PACHECK KAY SIR JAP KASI NIREVISE MO ULI</t>
   </si>
 </sst>
 </file>
@@ -783,7 +777,7 @@
         <v>56</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>57</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="72" x14ac:dyDescent="0.3">
@@ -870,7 +864,7 @@
         <v>55</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>58</v>
+        <v>37</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="64.2" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -897,7 +891,7 @@
         <v>39</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>57</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -907,9 +901,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1057,26 +1054,15 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BDD56014-E7AA-4ACA-8617-149CD20A7624}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67B8CFB1-3E32-4F77-BEE9-45E50532F813}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="6aee86ec-03d1-4b31-a311-732977dc0399"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1100,9 +1086,17 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67B8CFB1-3E32-4F77-BEE9-45E50532F813}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BDD56014-E7AA-4ACA-8617-149CD20A7624}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="6aee86ec-03d1-4b31-a311-732977dc0399"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update the value from the column `Saan pwede makita yung data?` and column `Status` for the spreadsheet `notes/Notes.xlsx`
</commit_message>
<xml_diff>
--- a/notes/Notes.xlsx
+++ b/notes/Notes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Visual_Studio_Codes\Data-Bank-System\notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C0EEC82-6AEF-440E-AF22-DE300DC9807E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{589DEEFE-087A-4D5C-B000-339E7E5404FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7B6336E8-B946-4BA0-8A65-45DEACE9975D}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="56">
   <si>
     <t>INDICATORS</t>
   </si>
@@ -150,9 +150,6 @@
     <t>DONE</t>
   </si>
   <si>
-    <t>PENDING</t>
-  </si>
-  <si>
     <t>Development Administration</t>
   </si>
   <si>
@@ -190,9 +187,6 @@
   </si>
   <si>
     <t>Peace and Order &amp; Public Safety</t>
-  </si>
-  <si>
-    <t>Sir Nico kaso nakaleave, nasa gilid siya, pwede naman daw ako gumawa muna ng initial ERD ko for that. May binigay na context sa akin si Sir Jap, naka time-based daw yung pag-track ng progress percentage ng mga master development plan and dapat tinatrack ko siya per barangay and not total barangay. Every 3 years dapat tinatrack ko yung progress percentage. Dapat din may 3 types of plans na sinasubmit bawat plan (Initial, Revised, Approved). Kung sakop pa ng range niya yung Date Range sa sinubmit na Plan, dapat updated yun</t>
   </si>
   <si>
     <r>
@@ -218,6 +212,9 @@
   </si>
   <si>
     <t>Binigay na sa akin yung data thru email</t>
+  </si>
+  <si>
+    <t>BINIGAY NA NIYA SA AKIN YUNG PAPER KUNG PAPAANO NILA MINEMEASURE YUNG DEVELOPMENT PLAN</t>
   </si>
 </sst>
 </file>
@@ -683,16 +680,16 @@
         <v>30</v>
       </c>
       <c r="G3" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="H3" s="3" t="s">
         <v>39</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>40</v>
       </c>
       <c r="I3" s="3" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="144" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
@@ -712,13 +709,13 @@
         <v>30</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="67.2" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -742,7 +739,7 @@
         <v>30</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H6" s="3" t="s">
         <v>35</v>
@@ -771,10 +768,10 @@
         <v>30</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="I7" s="3" t="s">
         <v>37</v>
@@ -782,28 +779,28 @@
     </row>
     <row r="10" spans="1:9" ht="72" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>41</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>42</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>25</v>
       </c>
       <c r="D10" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E10" s="4" t="s">
         <v>46</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>47</v>
       </c>
       <c r="F10" s="3" t="s">
         <v>30</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="I10" s="3" t="s">
         <v>37</v>
@@ -811,10 +808,10 @@
     </row>
     <row r="11" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>25</v>
@@ -826,13 +823,13 @@
         <v>25</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="I11" s="3" t="s">
         <v>37</v>
@@ -840,10 +837,10 @@
     </row>
     <row r="12" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>25</v>
@@ -855,13 +852,13 @@
         <v>25</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="I12" s="3" t="s">
         <v>37</v>
@@ -870,13 +867,13 @@
     <row r="13" spans="1:9" ht="64.2" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>25</v>
@@ -885,10 +882,10 @@
         <v>25</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I14" s="3" t="s">
         <v>37</v>
@@ -901,12 +898,9 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1054,15 +1048,26 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67B8CFB1-3E32-4F77-BEE9-45E50532F813}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BDD56014-E7AA-4ACA-8617-149CD20A7624}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="6aee86ec-03d1-4b31-a311-732977dc0399"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1086,17 +1091,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BDD56014-E7AA-4ACA-8617-149CD20A7624}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67B8CFB1-3E32-4F77-BEE9-45E50532F813}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="6aee86ec-03d1-4b31-a311-732977dc0399"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Added new row to the `notes/Notes.xlsx` spreadsheet
</commit_message>
<xml_diff>
--- a/notes/Notes.xlsx
+++ b/notes/Notes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Visual_Studio_Codes\Data-Bank-System\notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{589DEEFE-087A-4D5C-B000-339E7E5404FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{883F9928-B445-4DFA-A2AF-AF6B3C703C59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7B6336E8-B946-4BA0-8A65-45DEACE9975D}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="62">
   <si>
     <t>INDICATORS</t>
   </si>
@@ -215,6 +215,24 @@
   </si>
   <si>
     <t>BINIGAY NA NIYA SA AKIN YUNG PAPER KUNG PAPAANO NILA MINEMEASURE YUNG DEVELOPMENT PLAN</t>
+  </si>
+  <si>
+    <t>% improvement in government service delivery via social media</t>
+  </si>
+  <si>
+    <t>PIO</t>
+  </si>
+  <si>
+    <t>Social Media Programs</t>
+  </si>
+  <si>
+    <t>Use social media to target specific markets and improve public service engagement​</t>
+  </si>
+  <si>
+    <t>PENDING</t>
+  </si>
+  <si>
+    <t>Magtanong nalang kung papaano measurements nito</t>
   </si>
 </sst>
 </file>
@@ -589,7 +607,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6052A19D-DEF1-42F6-8C0B-B965C54104C1}">
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="85" style="2" customWidth="1"/>
@@ -891,6 +909,33 @@
         <v>37</v>
       </c>
     </row>
+    <row r="15" spans="1:9" ht="62.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="16" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="G16" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -898,12 +943,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C5A14CB71E5AFD41970DCC84E250D579" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="5cb02eec2b50f308d3d8c622b39c24e6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="6aee86ec-03d1-4b31-a311-732977dc0399" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3e885d23f01897dc3817344103bdb46e" ns3:_="">
     <xsd:import namespace="6aee86ec-03d1-4b31-a311-732977dc0399"/>
@@ -1047,6 +1086,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -1057,22 +1102,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BDD56014-E7AA-4ACA-8617-149CD20A7624}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="6aee86ec-03d1-4b31-a311-732977dc0399"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A5169A02-7206-4788-A357-046EDE3DF615}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1090,6 +1119,22 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BDD56014-E7AA-4ACA-8617-149CD20A7624}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="6aee86ec-03d1-4b31-a311-732977dc0399"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67B8CFB1-3E32-4F77-BEE9-45E50532F813}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Update the content from the `notes/Notes.xlsx`
</commit_message>
<xml_diff>
--- a/notes/Notes.xlsx
+++ b/notes/Notes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Visual_Studio_Codes\Data-Bank-System\notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{883F9928-B445-4DFA-A2AF-AF6B3C703C59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F56E6D4F-4929-41EB-8EF5-02B87C048457}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7B6336E8-B946-4BA0-8A65-45DEACE9975D}"/>
   </bookViews>
@@ -229,10 +229,10 @@
     <t>Use social media to target specific markets and improve public service engagement​</t>
   </si>
   <si>
-    <t>PENDING</t>
-  </si>
-  <si>
     <t>Magtanong nalang kung papaano measurements nito</t>
+  </si>
+  <si>
+    <t>DONE (INITIAL DESIGN KO LANG KAYA DI KO SURE IF TAMA)</t>
   </si>
 </sst>
 </file>
@@ -792,7 +792,7 @@
         <v>54</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>37</v>
+        <v>61</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="72" x14ac:dyDescent="0.3">
@@ -930,10 +930,10 @@
         <v>38</v>
       </c>
       <c r="H16" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="I16" s="3" t="s">
         <v>61</v>
-      </c>
-      <c r="I16" s="3" t="s">
-        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -943,6 +943,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C5A14CB71E5AFD41970DCC84E250D579" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="5cb02eec2b50f308d3d8c622b39c24e6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="6aee86ec-03d1-4b31-a311-732977dc0399" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3e885d23f01897dc3817344103bdb46e" ns3:_="">
     <xsd:import namespace="6aee86ec-03d1-4b31-a311-732977dc0399"/>
@@ -1086,35 +1101,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A5169A02-7206-4788-A357-046EDE3DF615}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67B8CFB1-3E32-4F77-BEE9-45E50532F813}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="6aee86ec-03d1-4b31-a311-732977dc0399"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1136,9 +1126,19 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67B8CFB1-3E32-4F77-BEE9-45E50532F813}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A5169A02-7206-4788-A357-046EDE3DF615}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="6aee86ec-03d1-4b31-a311-732977dc0399"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update the content of the `notes/Notes.xlsx`
</commit_message>
<xml_diff>
--- a/notes/Notes.xlsx
+++ b/notes/Notes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Visual_Studio_Codes\Data-Bank-System\notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F56E6D4F-4929-41EB-8EF5-02B87C048457}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E35A2D5-884B-4E28-9238-7176AF39E2D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7B6336E8-B946-4BA0-8A65-45DEACE9975D}"/>
   </bookViews>
@@ -211,9 +211,6 @@
     <t>running average. Injury count total in any injury types and severities</t>
   </si>
   <si>
-    <t>Binigay na sa akin yung data thru email</t>
-  </si>
-  <si>
     <t>BINIGAY NA NIYA SA AKIN YUNG PAPER KUNG PAPAANO NILA MINEMEASURE YUNG DEVELOPMENT PLAN</t>
   </si>
   <si>
@@ -229,10 +226,13 @@
     <t>Use social media to target specific markets and improve public service engagement​</t>
   </si>
   <si>
-    <t>Magtanong nalang kung papaano measurements nito</t>
-  </si>
-  <si>
-    <t>DONE (INITIAL DESIGN KO LANG KAYA DI KO SURE IF TAMA)</t>
+    <t>PENDING</t>
+  </si>
+  <si>
+    <t>Itatanong palang uli ni sir Jap, papaano nila minemeasure yun sa PIO</t>
+  </si>
+  <si>
+    <t>Pinasa na ni maam Joana thru email</t>
   </si>
 </sst>
 </file>
@@ -730,7 +730,7 @@
         <v>38</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="I4" s="3" t="s">
         <v>37</v>
@@ -789,10 +789,10 @@
         <v>38</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>61</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="72" x14ac:dyDescent="0.3">
@@ -912,16 +912,16 @@
     <row r="15" spans="1:9" ht="62.4" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="16" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="D16" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="E16" s="4" t="s">
         <v>58</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>59</v>
       </c>
       <c r="F16" s="3" t="s">
         <v>30</v>
@@ -933,7 +933,7 @@
         <v>60</v>
       </c>
       <c r="I16" s="3" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -943,21 +943,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C5A14CB71E5AFD41970DCC84E250D579" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="5cb02eec2b50f308d3d8c622b39c24e6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="6aee86ec-03d1-4b31-a311-732977dc0399" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3e885d23f01897dc3817344103bdb46e" ns3:_="">
     <xsd:import namespace="6aee86ec-03d1-4b31-a311-732977dc0399"/>
@@ -1101,10 +1086,35 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67B8CFB1-3E32-4F77-BEE9-45E50532F813}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A5169A02-7206-4788-A357-046EDE3DF615}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="6aee86ec-03d1-4b31-a311-732977dc0399"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1126,19 +1136,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A5169A02-7206-4788-A357-046EDE3DF615}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67B8CFB1-3E32-4F77-BEE9-45E50532F813}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="6aee86ec-03d1-4b31-a311-732977dc0399"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Modify the attributes of the table `system_implementations` and `system_reviews`. Convert to comment the table `system_status_history` table
</commit_message>
<xml_diff>
--- a/notes/Notes.xlsx
+++ b/notes/Notes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Visual_Studio_Codes\Data-Bank-System\notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E35A2D5-884B-4E28-9238-7176AF39E2D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B9344E9-6A7D-4564-9180-907E4302C6EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7B6336E8-B946-4BA0-8A65-45DEACE9975D}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="67">
   <si>
     <t>INDICATORS</t>
   </si>
@@ -233,6 +233,21 @@
   </si>
   <si>
     <t>Pinasa na ni maam Joana thru email</t>
+  </si>
+  <si>
+    <t>% increase in implementation of digital governance systems</t>
+  </si>
+  <si>
+    <t>PITO</t>
+  </si>
+  <si>
+    <t>PGB Systems</t>
+  </si>
+  <si>
+    <t>Implement systems such as eSig, Human Resources Information System (HRIS), Financial Management Information System (FMIS), and procurement system to enhance digital governance​</t>
+  </si>
+  <si>
+    <t>Nasusustain ba?</t>
   </si>
 </sst>
 </file>
@@ -607,7 +622,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6052A19D-DEF1-42F6-8C0B-B965C54104C1}">
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="85" style="2" customWidth="1"/>
@@ -933,6 +948,32 @@
         <v>60</v>
       </c>
       <c r="I16" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A18" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="G18" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="H18" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="I18" s="3" t="s">
         <v>59</v>
       </c>
     </row>
@@ -1087,18 +1128,18 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1120,6 +1161,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67B8CFB1-3E32-4F77-BEE9-45E50532F813}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BDD56014-E7AA-4ACA-8617-149CD20A7624}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
@@ -1133,12 +1182,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67B8CFB1-3E32-4F77-BEE9-45E50532F813}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Updated notes from the `notes/Notes.xlsx`
</commit_message>
<xml_diff>
--- a/notes/Notes.xlsx
+++ b/notes/Notes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Visual_Studio_Codes\Data-Bank-System\notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B9344E9-6A7D-4564-9180-907E4302C6EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16974FC6-9D79-4AEC-AEBA-8B575FE8A577}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7B6336E8-B946-4BA0-8A65-45DEACE9975D}"/>
   </bookViews>
@@ -247,7 +247,7 @@
     <t>Implement systems such as eSig, Human Resources Information System (HRIS), Financial Management Information System (FMIS), and procurement system to enhance digital governance​</t>
   </si>
   <si>
-    <t>Nasusustain ba?</t>
+    <t>Random day checking using API, so automated 'yun</t>
   </si>
 </sst>
 </file>
@@ -984,6 +984,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C5A14CB71E5AFD41970DCC84E250D579" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="5cb02eec2b50f308d3d8c622b39c24e6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="6aee86ec-03d1-4b31-a311-732977dc0399" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3e885d23f01897dc3817344103bdb46e" ns3:_="">
     <xsd:import namespace="6aee86ec-03d1-4b31-a311-732977dc0399"/>
@@ -1127,15 +1136,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
@@ -1143,6 +1143,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67B8CFB1-3E32-4F77-BEE9-45E50532F813}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A5169A02-7206-4788-A357-046EDE3DF615}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1156,14 +1164,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67B8CFB1-3E32-4F77-BEE9-45E50532F813}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Update the content of the notes spreadsheet
</commit_message>
<xml_diff>
--- a/notes/Notes.xlsx
+++ b/notes/Notes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Visual_Studio_Codes\Data-Bank-System\notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16974FC6-9D79-4AEC-AEBA-8B575FE8A577}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C03B01BB-9C10-4E71-97E4-7A4EA371CBF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7B6336E8-B946-4BA0-8A65-45DEACE9975D}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="68">
   <si>
     <t>INDICATORS</t>
   </si>
@@ -248,6 +248,9 @@
   </si>
   <si>
     <t>Random day checking using API, so automated 'yun</t>
+  </si>
+  <si>
+    <t>PENDING PERO NAKASTORE NA SA DBML NATIN</t>
   </si>
 </sst>
 </file>
@@ -974,7 +977,7 @@
         <v>66</v>
       </c>
       <c r="I18" s="3" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -984,15 +987,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C5A14CB71E5AFD41970DCC84E250D579" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="5cb02eec2b50f308d3d8c622b39c24e6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="6aee86ec-03d1-4b31-a311-732977dc0399" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3e885d23f01897dc3817344103bdb46e" ns3:_="">
     <xsd:import namespace="6aee86ec-03d1-4b31-a311-732977dc0399"/>
@@ -1136,6 +1130,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
@@ -1143,14 +1146,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67B8CFB1-3E32-4F77-BEE9-45E50532F813}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A5169A02-7206-4788-A357-046EDE3DF615}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1164,6 +1159,14 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67B8CFB1-3E32-4F77-BEE9-45E50532F813}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>